<commit_message>
handle error temp image phhash
</commit_message>
<xml_diff>
--- a/storage/assets/webc_excel/11_2025/WEBC LIMA UTAMA (Start Juni 2025).xlsx
+++ b/storage/assets/webc_excel/11_2025/WEBC LIMA UTAMA (Start Juni 2025).xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pkscindy0050\Desktop\KPB Done\WEBC Sementara\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willi\Project\cek-gambar-astras\storage\assets\webc_excel\11_2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EBF8804-07A4-4899-AA34-4AFDA75387B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7500"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,13 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="36">
-  <si>
-    <t>Tidak ada WEBC JUNI 2025</t>
-  </si>
-  <si>
-    <t>Tidak ada WEBC JULI 2025</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="34">
   <si>
     <t>nama_region</t>
   </si>
@@ -138,7 +133,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -456,129 +451,119 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:R2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:18" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q3" s="1" t="s">
+    <row r="2" spans="1:18" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="R3" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="4" spans="1:18" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="L2" s="1">
+        <v>5080</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="L4" s="1">
-        <v>5080</v>
-      </c>
-      <c r="M4" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="N4" s="1" t="s">
+      <c r="P2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="O4" s="1" t="s">
+      <c r="Q2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="P4" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="R4" s="1">
+      <c r="R2" s="1">
         <v>0</v>
       </c>
     </row>
@@ -588,117 +573,117 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="M1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="N1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="O1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="P1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="Q1" t="s">
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>18</v>
       </c>
-      <c r="R1" t="s">
+      <c r="B2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="C2" t="s">
         <v>20</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>21</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>22</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>23</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>24</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>25</v>
       </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
         <v>26</v>
       </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
         <v>27</v>
       </c>
-      <c r="I2" t="s">
+      <c r="K2" t="s">
         <v>28</v>
-      </c>
-      <c r="J2" t="s">
-        <v>29</v>
-      </c>
-      <c r="K2" t="s">
-        <v>30</v>
       </c>
       <c r="L2">
         <v>5080</v>
       </c>
       <c r="M2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N2" t="s">
+        <v>30</v>
+      </c>
+      <c r="O2" t="s">
         <v>31</v>
       </c>
-      <c r="N2" t="s">
+      <c r="P2" t="s">
         <v>32</v>
       </c>
-      <c r="O2" t="s">
+      <c r="Q2" t="s">
         <v>33</v>
-      </c>
-      <c r="P2" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>35</v>
       </c>
       <c r="R2">
         <v>0</v>

</xml_diff>